<commit_message>
Text agent - colab
</commit_message>
<xml_diff>
--- a/COLAB/results.xlsx
+++ b/COLAB/results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1943,6 +1943,1273 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>phi3:mini</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>After beam come back from long beam dump what to do</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>1. Check the current (CERS)
+2. After IC1 stabilized
+3. Open the shutter 'opens'
+4. Check the IC1
+5. If you have little counts at IC1, follow these steps: press 3 in stkechy_mostab and use mostab to go maximum IC2; then proceed to maximum IC1 by pressing 1 in stkechy_mostab</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>llama2:latest</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>After beam come back from long beam dump what to do</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Based on the provided context, the steps to take after the beam comes back from a long beam dump are as follows:
+1. Check the current (CERS)
+2. After IC1 stabilized, open the shutter 'opens'
+3. Check the IC1
+4. If you have little counts at IC1, follow the below steps (if not, consult the beamline scientist):
+	* Step 5: Press 3 in stkechy_mostab
+	* Step 6: Use mostab to go to maximum IC2
+	* Step 7: Go to maximum IC1
+	* Step 8: Press 1 in stkechy_mostab
+Additionally, it is mentioned that data policy states that raw data is stored for six months and processed data is stored for a year. If you need more time, consult the beamline scientist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>deepseek-r1:1.5b</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>After beam come back from long beam dump what to do</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>After the beam has returned from the long beam dump, follow these steps:
+1. **Check CERS**: Ensure the current conditions are correct for your experiment.
+2. **IC1 Stabilized**: Confirm that IC1 is properly stabilized to avoid any issues.
+3. **Shutter Opening**: Open the shutter as specified to allow proper ionization.
+4. **IC1 Check**: Verify the state of IC1 after these steps.
+5. **Little Counts Handling**:
+   - If there are little counts at IC1, proceed with:
+     a. Press 3 in stkechy_mostab
+     b. Use mostab go maximum IC2
+     c. Go to maximum IC1
+     d. Press 1 in stkechy_mostab
+This sequence ensures all necessary adjustments and operations are performed correctly after the beam dump.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>gemma:2b</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>After beam come back from long beam dump what to do</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Sure, here's the answer to the question:
+After beam come back from long beam dump, the following steps should be followed:
+1. Check the current (CERS)
+2. After IC1 stabilized
+3. Open the shutter 'opens'
+4. Check the IC1
+5. If you have little counts at IC1 follow the below steps:
+    - Stop the experiment
+    - Talk to beamline scientist</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>deepseek-coder:6.7b</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>After beam come back from long beam dump what to do</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Check the current (CERS)
+2. After IC1 stabilized 
+3. Open the shutter 'opens' 
+4. Check the IC1
+5. If you have little counts at IC1, follow these steps:
+   - Press 3 in stkechy_mostab
+   - Use mostab go maximum IC2
+   - Go to maximum IC1 
+   - Press 1 in stkechy_mostab
+6. Transfer the data using Globus or other file transfer tools. The processed data can be found on id4baux server. If you need more time, consult your beamline scientist.
+7. If you have a lower diode signal, follow these steps: 
+   - Stop the experiment
+   - Talk to the beamline scientist
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>codellama:7b-instruct</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>After beam come back from long beam dump what to do</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+After the beam comes back from a long beam dump, there are several steps that need to be taken to ensure proper operation of the synchrotron beamline. These steps include:
+1. Checking the current (CERS)
+2. After IC1 stabilized
+3. Opening the shutter 'opens'
+4. Checking the IC1
+5. If you have little counts at IC1, follow the below steps (if not, talk to the beamline scientist):
+6. Press 3 in stkechy_mostab
+7. Use mostab go maximum IC2
+8. Go to maximum IC1
+9. Press 1 in stkechy_mostab
+It is important to note that these steps are specific to the ID4B beamline and may vary depending on the specific requirements of your experiment. It is recommended to consult with a beamline scientist or engineer for guidance on any issues related to beamline operation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>mistral:instruct</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>After beam come back from long beam dump what to do</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> After a long beam dump, follow these steps:
+1. Check the current (CERS)
+2. Wait for IC1 to stabilize
+3. Open the shutter 'opens'
+4. Check the IC1
+5. If you have little counts at IC1, proceed with the following steps:
+   a. Press 3 in stkechy_mostab
+   b. Use mostab to go to maximum IC2
+   c. Go to maximum IC1
+   d. Press 1 in stkechy_mostab
+6. If you have signal, some values at IC1:
+   a. Proceed with the experiment using macros and 'batches' (refer to the SPEC manual pymca.pdf)
+7. If you have a lower diode signal:
+   a. Stop the experiment
+   b. Talk to the beamline scientist</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>After beam come back from long beam dump what to do</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> After a long beam dump, follow these steps:
+1. Check the current (CERS)
+2. Wait for IC1 to stabilize
+3. Open the shutter 'opens'
+4. Check the IC1
+5. If you have little counts at IC1:
+    - Process the data and copy it to your server
+    - If you need more time, consult your beamline scientist
+    - Press 3 in stkechy_mostab
+    - Use mostab to go to maximum IC2
+    - Go to maximum IC1
+    - Press 1 in stkechy_mostab
+6. If you have signal and some values at IC1:
+    - Press 3 in stkechy_mostab
+    - Use mostab to go to maximum IC2
+    - Go to maximum IC1
+    - Press 1 in stkechy_mostab
+If you encounter a lower diode signal, stop the experiment and talk to the beamline scientist. To transfer data, use globus. The data is stored at id4baux after processing. If you need help or have questions about data recovery or location, consult your beamline scientist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>phi3:mini</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>show Raw data visulization software</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Raw data visualization software is available. It can be used to produce rudimentary plots of the raw data on a printer at the end of each scan and also for real-time plotting during scans, as indicated in various sources such as /home/vallurs/research/data/md_files/beamline_basics.md and nexpy documentation (https://nexpy.github.io/nexpy/pythongui.html).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>llama2:latest</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>show Raw data visulization software</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Based on the provided context, the answer to your question is:
+Raw data visualization software is available in the following packages:
+1. Nexpy - A Python-based data visualization package that provides various tools for stacking raw data and customizing the environment for specialized requirements.
+2. Data Basics - A package that provides capabilities for screen 6, including data visualization software.
+3. ID4B - A code that provides various tools for stacking raw data and customizing the environment for specialized requirements.
+These packages can be accessed through the following links:
+* Nexpy: [https://nexpy.github.io/nexpy/pythongui.html](https://nexpy.github.io/nexpy/pythongui.html)
+* Data Basics: [https://raw-data-visualization.readthedocs.io/en/latest/](https://raw-data-visualization.readthedocs.io/en/latest/)
+* ID4B: [https://drive.google.com/drive/folders/1376859027?usp=sharing](https://drive.google.com/drive/folders/1376859027?usp=sharing)
+Please note that the provided links are the most up-to-date sources of information and may be subject to change over time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>deepseek-r1:1.5b</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>show Raw data visulization software</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>The source that mentions "raw data visualization software" is /home/vallurs/research/data/md_files/beamline_basics.md, specifically screen 6 which includes a figure with "Data' visualization package." However, this does not directly refer to raw data visualization software. The document discusses tools for beamline control and data processing rather than software itself.
+**Answer:** There is no direct mention of raw data visualization software in the provided context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>gemma:2b</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>show Raw data visulization software</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Sure, here is the raw data visulization software.
+[Image title](https://github.com/suchismitasarker/CHESS-ID4B-QM2/blob/main/pictures/Screen6.png?raw=true){ width="600" }</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>deepseek-coder:6.7b</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>show Raw data visulization software</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Based on the provided context and question, it seems you are looking for a way to visualize raw data. The screenshots in your documents suggest that there might be a possibility of using a raw data visualization software like Nexpy or Matplotlib in Python. 
+Nexpy is a python package for interactive scientific computing which can handle large datasets and provides various tools for stacking the raw data, but it's not clear from your context if you need this kind of functionality. If you do, you might want to check out their documentation at https://nexpy.github.io/nexpy/pythongui.html
+Matplotlib is a plotting library for Python that can create static, animated, and interactive visualizations in Python. It's widely used in scientific computing and data analysis. You might find it useful if you need more advanced features like 3D plots or time series analysis. Here's an example of how to use Matplotlib:
+```python
+import matplotlib.pyplot as plt
+import numpy as np
+# Create some data
+x = np.linspace(0, 2 * np.pi, 400)
+y = np.sin(x ** 2)
+plt.figure()
+plt.plot(x, y)
+plt.show()
+```
+Please note that both Nexpy and Matplotlib are powerful tools but they require some knowledge of Python programming to use effectively. If you're not familiar with these or any other programming languages, consider learning them before using these tools.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>codellama:7b-instruct</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>show Raw data visulization software</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+The raw data visualization software is Nexpy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>mistral:instruct</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>show Raw data visulization software</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The raw data visualization software available is mentioned in the provided context as follows:
+* From the file /home/vallurs/research/data/md_files/beamline_basics.md, it is stated that a raw data visualization software is used.
+* In the same file, it is also hinted that Screen 6 contains this software.
+* The file /home/vallurs/research/data/drive_docs/spec Manual cambria.pdf mentions that a rudimentary plot can be produced on the screen using the command 'splot'.
+* It is also recommended to take a look at the data visualization package Nexpy, which can be found in the documentation at this link: [Nexpy visulization Documentation](https://nexpy.github.io/nexpy/pythongui.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>show Raw data visulization software</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The provided context mentions two raw data visualization software options:
+1. A software mentioned in the file `/home/vallurs/research/data/md_files/beamline_basics.md` but no specific name is given. (You can find a screenshot of Screen 6 from this file which might give you more information.)
+2. Nexpy, a data visualization package recommended in the file `/home/vallurs/research/data/md_files/nexpy.md`. You can find documentation for Nexpy at [Nexpy visulization Documentation](https://nexpy.github.io/nexpy/pythongui.html).
+For more information, you may want to check the files mentioned above or consult with the researcher who created these documents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>phi3:mini</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Provide the macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>```bash
+for (loopT=325; loopT&lt;476; loopT+=25){
+    eval(sprintf("threextalscan %d 180", loopT))
+}
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>llama2:latest</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Provide the macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Not found in the provided documents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>deepseek-r1:1.5b</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Provide the macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Tscans_low_to_high_N2</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>gemma:2b</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Provide the macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Sure, here is the macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen:
+```python
+# Temperature Dependent scan: 300K- 475K at 25K temperature interval
+def Tscans_high_N2 '
+te = 325
+for (loopT=325; loopT&lt;476; loopT=loopT+25){
+    eval(sprintf("threextalscan %s 180",loopT))
+}
+# Temperature Dependent scan: 90K- 300K at 25K temperature interval
+def Tscans_low_to_high_N2 '
+for (loopT=90; loopT &lt; 301; loopT=loopT+15){
+    eval(sprintf("threextalscan %s 180", loopT))
+}
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>deepseek-coder:6.7b</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Provide the macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is a simple example of how you can perform a temperature scan from 300K to 475K with an interval of 25K using the `threextalscan` command in Synchrotron beamline control system. This script assumes that you are already familiar with the basic commands and syntax for controlling the instrument:
+```python
+te = 300 # Initial temperature
+for loopT in range(300, 476, 25): # Loop from 300K to 475K at intervals of 25K
+    eval(f"threextalscan {loopT} 180") # Perform a reciprocal space scan with the current temperature
+```
+This script sets the initial temperature (`te = 300`) and then loops over each temperature from `300K` to `475K` in steps of `25K`. For each iteration, it executes the `threextalscan` command with the current temperature and a scan time of `180` seconds.
+Please note that you need to replace `"threextalscan"` with your actual command for reciprocal space scans if they are different in your system. Also, ensure that the temperatures are set correctly according to your instrument's capabilities and safety guidelines.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>codellama:7b-instruct</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Provide the macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+The macro for temperature-dependent scans from 300K to 475K at a 25K interval under nitrogen is as follows:
+```scss
+def TScans_high_N2 '
+te = 325
+for (loopT=325; loopT&lt;476; loopT=loopT+25){
+eval(sprintf("threextalscan %s 180",loopT))
+}
+```
+This macro sets the temperature to 325K, and then loops through a range of temperatures from 325K to 476K with an interval of 25K. For each temperature, it runs the `threextalscan` command with the current temperature value and exposure time of 180 seconds.
+Note that this macro assumes that you have already set up the temperature switches in your system to control the temperature between 300K and 475K under nitrogen. If you need to modify these standard macros to suit your specific needs, please refer to the documentation for your specific instrument or consult with a qualified technician.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>mistral:instruct</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Provide the macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The provided context contains a macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen, named `TScans_high_N2`. Here is the macro:
+```bash
+def TScans_high_N2 '
+te = 325
+for (loopT=325; loopT&lt;476; loopT=loopT+25){
+eval(sprintf("threextalscan %s 180",loopT))
+}
+'
+```
+This macro sets the temperature to 325K (which is 55°C) and then performs a series of scans from 325K to 475K at an interval of 25K. The `threextalscan` command is used for performing reciprocal space scans, and the number following it represents the temperature in Kelvin. The last argument specifies the number of frames per second during the scan. In this case, it's set to 180.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Provide the macro for temperature dependent scans from 300K to 475K at 25K interval under nitrogen</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The provided context includes a macro named `TScans_high_N2` that performs a temperature-dependent scan from 300K to 475K at 25K interval under nitrogen. Here is the macro:
+```bash
+def TScans_high_N2 '
+te = 325
+for (loopT=325; loopT&lt;476; loopT=loopT+25){
+eval(sprintf("threextalscan %s 180",loopT))
+}
+'
+```
+This macro initializes the temperature to 325K, then iterates through temperatures from 325K to 475K in increments of 25K, and runs a `threextalscan` with an angle of 180 degrees for each temperature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>phi3:mini</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>How to Create file structure for  single crystal sample alignment - HDRM</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>a. FOURC&gt; newfile &lt;samplename&gt;  
+b. samplename should be chemical name of your sample, make sure you created folder in your directory   
+c. Open the script named 'HDRMscans.mac' and sort out your path using command 'sortmypathout'.    
+d. In the HDRMscans.mac file find _mysample = &lt;sample_identifier&gt; change it to reflect your sample identifier  
+e. Save changes in the document</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>llama2:latest</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>How to Create file structure for  single crystal sample alignment - HDRM</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>The provided context provides information on how to create a file structure for single crystal sample alignment using the HDRM software. Here is a direct answer to your question:
+To create a file structure for single crystal sample alignment - HDRM, follow these steps:
+1. Create a newfile as FOURC&gt;newfile &lt;samplename&gt;. Replace &lt;samplename&gt; with the chemical name of your sample.
+2. Open the HDRMscans.mac script and sort your path (sortmypathout).
+3. Change the _mysample = &lt;sample_identifier&gt; where _mysample is the sample identifier.
+4. Save the file.
+Note: The provided context also mentions basic steps for single crystal thin-film sample alignment - HDRM, but these steps are not relevant to creating a file structure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>deepseek-r1:1.5b</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>How to Create file structure for  single crystal sample alignment - HDRM</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Creating the file structure for single crystal sample alignment - HDRM involves setting up directories, defining samplename, and organizing data effectively. Here are the steps:
+1. Create a newfile with the samplename specified in your document.
+2. Define the samplename as the chemical name of your sample, ensuring you create the necessary folder structure.
+3. Open the HDRMscans.mac script and sort your path (sortmypathout).
+4. Change the _mysample identifier to the sample identifier used in your document.
+5. Save the file with these settings.
+These steps ensure proper organization for data management within the HDRM system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>gemma:2b</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>How to Create file structure for  single crystal sample alignment - HDRM</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Sure, here's how to create the file structure for single crystal sample alignment - HDRM:
+**Step 1:** Create newfile as FOURC&gt;newfile &lt;samplename&gt;
+**Step 2:** Create newfile as FOURC&gt;newfile &lt;samplename&gt;
+**Step 3:** Open HDRMscans.mac script and sort your path (sortmypathout)
+**Step 4:** Save the file</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>deepseek-coder:6.7b</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>How to Create file structure for  single crystal sample alignment - HDRM</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">To create a file structure for single crystal sample alignment - HDRM, you need to follow these steps:
+1. **Create newfile**: This command is used in FOURC to create a new file with the specified name. The syntax is `FOURC&gt;newfile samplename` where "samplename" is the name of your sample. 
+2. **Sample Name**: Choose a unique identifier for your sample and make sure you have created a folder in your directory with this name. This will be used as the file path to store data related to this sample.
+3. **Open HDRMscans.mac script**: The .mac (Macro) scripts are used to control the operation of the beamline. Open the `HDRMscans.mac` script and sort your path using the command `sortmypathout`. This will ensure that all necessary files and directories are included in the search path.
+4. **Change Sample Identifier**: In the HDRMscans.mac script, change the value of _mysample to match the sample identifier you have chosen for your sample. The line should look like this `_mysample = &lt;sample_identifier&gt;` where "&lt;sample_identifier&gt;" is the unique name you chose for your sample.
+5. **Save File**: After making these changes, save the HDRMscans.mac script. This will ensure that your changes are saved and can be used in future operations of the beamline.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>codellama:7b-instruct</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>How to Create file structure for  single crystal sample alignment - HDRM</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+To create a file structure for single crystal sample alignment using HDRM, follow these steps:
+1. Open the terminal and navigate to the directory where you want to store your data.
+2. Use the command `FOURC&gt;newfile &lt;samplename&gt;` to create a new file with the name `&lt;samplename&gt;`.
+3. Use the command `FOURC&gt;umvr samz2 0.1` to set the relative motion of the sample movement up (+) and down (-).
+4. Use the command `FOURC&gt;umv phi2 0` to set the rotation angle of the sample around the z-axis to 0 degrees.
+5. Use the command `FOURC&gt;umv phi2 180` to set the rotation angle of the sample around the z-axis to 180 degrees.
+6. Move the x and y axes to make the sample position match the cursor.
+7. Use the command `FOURC&gt;umv phi2 90` to rotate the sample around the z-axis by 90 degrees.
+8. Use the command `FOURC&gt;umv phi2 270` to rotate the sample around the z-axis by 270 degrees.
+9. Repeat steps 6 and 7 until the center of the axis matches the sample position.
+10. Save the file with the name `&lt;samplename&gt;` using the command `FOURC&gt;save`.
+Note: Make sure to replace `&lt;samplename&gt;` with the actual name of your sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>mistral:instruct</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>How to Create file structure for  single crystal sample alignment - HDRM</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> To create a file structure for single crystal sample alignment in HDRM, follow these steps:
+1. Open the FourCC console by typing `FOURC` in the terminal.
+2. Create a new file using the command `newfile &lt;samplename&gt;`, where `&lt;samplename&gt;` is the chemical name of your sample. Make sure you have created a folder with the same name in your directory.
+3. Open the HDRMscans.mac script and sort your path by executing the command `sortmypathout`.
+4. Change the sample identifier in the line `_mysample = &lt;sample_identifier&gt;` where `&lt;sample_identifier&gt;` is the name you have given to your sample.
+5. Save the file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>How to Create file structure for  single crystal sample alignment - HDRM</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> To create a file structure for single crystal sample alignment - HDRM, follow these steps:
+1. Open the FourC command line interface.
+2. Create a new file using the following command: `FOURC&gt;newfile &lt;samplename&gt;`
+   Replace `&lt;samplename&gt;` with the chemical name of your sample. Make sure you have created a folder in your directory with the same name as the sample.
+3. Open the HDRMscans.mac script and sort your path by using the command: `sortmypathout`
+4. Change the _mysample = &lt;sample_identifier&gt; where _mysample is the sample identifier.
+5. Save the file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>phi3:mini</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Names of the six-circle Huber Diffractometer's motor</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>&lt;b&gt;Table 1&lt;/b&gt;: Names of the six-circle Huber Diffractometer's motor
+Source: /home/vallurs/research/data/md_files/diffractometer.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>llama2:latest</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Names of the six-circle Huber Diffractometer's motor</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Based on the provided context, the names of the six-circle Huber Diffractometer's motor are:
+1. Alpha
+2. Beta
+3. Azimuth
+4. Omega
+5. Lambda
+6. Phi</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>deepseek-r1:1.5b</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Names of the six-circle Huber Diffractometer's motor</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>The names of the six-circle Huber Diffractometer's motor are listed in Table 1 of /home/vallurs/research/data/md_files/diffractometer.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>gemma:2b</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Names of the six-circle Huber Diffractometer's motor</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Sure, here is the requested information from the context:
+The names of the six-circle Huber Diffractometer's motor are not explicitly mentioned in the context, so I cannot extract the requested information from the context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>deepseek-coder:6.7b</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Names of the six-circle Huber Diffractometer's motor</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The names of the six-circle Huber Diffractometer's motors are not explicitly stated in the provided context. However, based on the information given, it seems that the motors involved might include:
+1. Sample orientation (alpha)
+2. Detector orientation (beta)
+3. Azimuthal rotation (gamma)
+4. Omega angle (fourth motor)
+5. Lambda angle (fifth motor)
+6. Chi angle (sixth motor)
+Please refer to the specific manuals or documentation for more detailed information about these motors and their naming conventions.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>codellama:7b-instruct</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Names of the six-circle Huber Diffractometer's motor</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+The names of the six-circle Huber diffractometer's motors are shown in Table 1 below. The table is taken from the reference [1] and [2].
+| Motor Name | Description |
+| --- | --- |
+| m1 | Sample rotation motor |
+| m2 | Detector rotation motor |
+| m3 | Sample translation motor |
+| m4 | Detector translation motor |
+| m5 | Sample inclination motor |
+| m6 | Detector inclination motor |
+Note that the names of the motors may vary depending on the specific diffractometer and its configuration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>mistral:instruct</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Names of the six-circle Huber Diffractometer's motor</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The names of the six-circle Huber Diffractometer's motor are not explicitly listed in the provided context. However, they are shown in Table 1 which is available at /home/vallurs/research/data/md_files/diffractometer.md. You can access and view the table from this location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Names of the six-circle Huber Diffractometer's motor</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The names of the six-circle Huber Diffractometer's motor are not explicitly listed in the provided context. However, they are mentioned to be shown in Table 1 which is available at /home/vallurs/research/data/md_files/diffractometer.md. Therefore, you can find the names of the motors by accessing and reading Table 1 from that file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>phi3:mini</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If you lost fourc/SPEC terminal </t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>1. Open a new terminal and type `findspec`. If SPEC is open, it will take you to the SPEC terminal automatically. Skip below steps if this happens. Otherwise proceed with step two as described in Instruction 2 of your document for further assistance on opening or accessing the lost fourc/SPEC terminal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>llama2:latest</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If you lost fourc/SPEC terminal </t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>The steps to follow if you lost the fourc/SPEC terminal are as follows:
+Step 1: Open a new terminal window and type `fourc`. If SPEC is open, it will go to the SPEC terminal. Skip the below steps.
+Step 2: Check the getPid number (you do not have to do this step).
+Step 3: Type `fg &lt;getPid number&gt;` (example # fg 21192) (you do not have to do this step).
+If SPEC is still missing, talk to a beamline scientist. If you change the spec current directory, you can reference open files either by the file name or the getPid number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>deepseek-r1:1.5b</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If you lost fourc/SPEC terminal </t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Step 1: Open a new terminal  
+Step 2: Type `findspec` (it will provide all the spec information)  
+Answer:
+If you lost fourc/SPEC terminal, open a new terminal and type `findspec`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>gemma:2b</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If you lost fourc/SPEC terminal </t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Sure, here's the answer to the question:
+**STEP 1: If you lost fourc/SPEC terminal**
+* Open terminal
+* Type `findspec` (it will provide all the spec information)
+* If SPEC is open it will go to the SPEC terminal
+* Skip the below steps</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>deepseek-coder:6.7b</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If you lost fourc/SPEC terminal </t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">To recover a lost SPEC (Special Program for Experiments in Coherent Radiation) terminal, follow these steps:
+1. Open a new terminal and type `fourc` to start the SPEC program. If it's not working as expected or if you can't find the SPEC terminal, then proceed with the following steps.
+2. If `quit` doesn't work, try using `kill -9 &lt;getPid number&gt;` command where `&lt;getPid number&gt;` is the process ID of the SPEC program. This will forcefully terminate the SPEC program if it's running in the background.
+3. Open a new terminal and type `findspec` to find all instances of SPEC running on your system. If SPEC is still open, you can directly go to its terminal without performing any further steps.
+4. If SPEC is not found or if it's still missing after the above steps, contact the beamline scientist and explain the situation. They might be able to guide you through recovering the lost terminal. 
+Please note that these instructions are based on general knowledge about how to start and stop SPEC programs in Linux systems. The exact commands may vary depending on your specific system configuration. Always refer to official documentation or support resources for precise instructions.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>codellama:7b-instruct</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If you lost fourc/SPEC terminal </t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+To regain access to the fourc/SPEC terminal, follow these steps:
+1. Open a new terminal.
+2. Type `fourc` and press Enter. If you don't find the SPEC terminal, then type `quit` and press Enter.
+3. Type `fourc` again and press Enter.
+4. If you still can't access the SPEC terminal, try typing `kill -9 &lt;getPid number&gt;` (example: `kill -9 21192`) and then open a new terminal and type `fourc`.
+5. If you don't find anythng after step 4, talk to the beamline scientist or check the getPid number (you do not have to do this step).
+6. Check the getPid number (you do not have to do this step) and type `fg &lt;getPid number&gt;` (example: `fg 21192`) and press Enter.
+7. If you still can't access the SPEC terminal, try checking the news file (you do not have to do this step).
+8. Check the news file (you do not have to do this step) and type `reconfig` and press Enter.
+9. Install macros (you do not have to do this step).
+10. Install /usr/local/lib/spec.d/standard.mac (you do not have to do this step).
+11. Install /usr/local/lib/spec.d/four.mac (you do not have to do this step).
+12. Install the high res graphics filters (you do not have to do this step).
+13. Install help files (you do not have to do this step).
+14. Clear out old help files (you do not have to do this step).
+15. Make the "help" help file (you do not have to do this step).
+16. Copying help files (you do not have to do this step).
+17. Changing ownership of help files to gerry (you do not have to do this step).
+18. Installing the chelp program (you do not have to do this step).
+19. Installing the show_state program (you do not have to do this step).
+20. Installing data_pipe auxiliary files (you do not have to do this step).</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>mistral:instruct</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If you lost fourc/SPEC terminal </t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> To regain access to the fourc/SPEC terminal, follow these steps in order:
+1. Open a new terminal.
+2. Type `fourc` in the terminal.
+If the SPEC terminal does not open, perform the following steps:
+1. In the same terminal, type `quit`.
+2. Again, type `fourc`.
+If the SPEC terminal still does not open, try the following:
+1. Open a new terminal.
+2. Type `findspec` in the terminal. This command will provide all the spec information. If SPEC is open, it will go to the SPEC terminal. Skip the below steps if this happens.
+3. Check the getPid number (you do not have to do this step).
+4. Type `fg &lt;getPid number&gt;` in the terminal (example: fg 21192). You do not have to do this step.
+If you still cannot find the SPEC terminal, contact a beamline scientist for assistance. If necessary, use the command `kill -9 &lt;getPid number&gt;` (example: kill -9 21192) to terminate any running SPEC processes and then open a new terminal and type `fourc`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If you lost fourc/SPEC terminal </t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> To regain access to the fourc/SPEC terminal, follow these steps:
+1. Open a new terminal.
+2. Type `fourc` in the terminal.
+If the SPEC terminal does not open, try the following:
+1. Open a new terminal.
+2. Type `findspec` in the terminal. This will provide all the spec information. If SPEC is open, it will go to the SPEC terminal. Skip the below steps if this happens.
+3. Check the getPid number (you do not have to do this step).
+4. If you still cannot find the SPEC terminal, type `kill -9 &lt;getPid number&gt;` (example: `kill -9 21192`) in a new terminal and then type `fourc`.
+If nothing works after these steps, contact the beamline scientist for assistance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>phi3:mini</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>what command for setting the temperature?</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>```plaintext
+settemp
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>llama2:latest</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>what command for setting the temperature?</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Based on the provided context, the command for setting the temperature is "settemp".</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>deepseek-r1:1.5b</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>what command for setting the temperature?</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>The correct command for setting the temperature is:
+**settemp**
+This command serves as a primary tool for adjusting the temperature in the system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>gemma:2b</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>what command for setting the temperature?</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>The command for setting the temperature is:
+```
+settemp # Set the temperature
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>deepseek-coder:6.7b</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>what command for setting the temperature?</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The command for setting the temperature in both Chunk 4 and Chunk 6 is "settemp".
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>codellama:7b-instruct</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>what command for setting the temperature?</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+The answer to your question is "settemp".</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>mistral:instruct</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>what command for setting the temperature?</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The command for setting the temperature is 'settemp'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>what command for setting the temperature?</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The command for setting the temperature is 'settemp'.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>